<commit_message>
@espark-asim  JS05B-10P-100-3-4 Ribbon cable update in USM BOM
</commit_message>
<xml_diff>
--- a/Design-Files/OFP_USM_v1.5/BOM/Client-BOM-OFP_USM_v1.5.xlsx
+++ b/Design-Files/OFP_USM_v1.5/BOM/Client-BOM-OFP_USM_v1.5.xlsx
@@ -264,16 +264,16 @@
     <t>Peripheral</t>
   </si>
   <si>
-    <t>0.3mm 10P 0.5mm 60mm P=0.5mm FFC Cable (Flexible Flat Cable) ROHS</t>
-  </si>
-  <si>
     <t>P=0.5mm</t>
   </si>
   <si>
-    <t>AB03A0100000180A</t>
-  </si>
-  <si>
-    <t>BZCN</t>
+    <t>JS05B-10P-100-3-4</t>
+  </si>
+  <si>
+    <t>JUSHUO</t>
+  </si>
+  <si>
+    <t>0.3mm 10P 0.5mm Reverse 10cm P=0.5mm FFC Cable (Flexible Flat Cable) ROHS</t>
   </si>
 </sst>
 </file>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="K15" s="7"/>
     </row>
-    <row r="16" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="11">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1255,16 +1255,16 @@
         <v>79</v>
       </c>
       <c r="E16" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="F16" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="F16" s="9" t="s">
+      <c r="G16" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="G16" s="10" t="s">
+      <c r="H16" s="9" t="s">
         <v>83</v>
-      </c>
-      <c r="H16" s="9" t="s">
-        <v>84</v>
       </c>
       <c r="I16" s="10" t="s">
         <v>79</v>

</xml_diff>